<commit_message>
Fix IZZ/Refugee naming consistency and guard visualize edge cases
Correct demo case variable names after the abbreviations were written out in full:
- Refugee: add the missing underscore in the LanguageAcquisitionUkrainians_Integration_* suffixes
- Refugee: fix AccesToTransport -> AccessToTransport typo
- IZZ: collapse the double underscore PhysicalStrainReduction__ -> PhysicalStrainReduction_

Guard visualize.py against two edge cases:
- theme_weight pie chart: return 0 (with an English warning) instead of raising
  ZeroDivisionError when a theme's total relative key output weight is 0; the legend
  percentage calculation is guarded the same way
- _create_appreciation_graph: warn and return early when called before .appreciate()
  has populated appreciation_functions, instead of the generic "'<key>' is not a valid option"

Applied consistently across the csv, json and xlsx representations.

Refs #114, #131

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/vlinder/data/IZZ/xlsx/IZZ.xlsx
+++ b/src/vlinder/data/IZZ/xlsx/IZZ.xlsx
@@ -2431,7 +2431,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2441,7 +2441,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2451,7 +2451,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2461,7 +2461,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2631,7 +2631,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2641,7 +2641,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2651,7 +2651,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2661,7 +2661,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -2831,7 +2831,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2841,7 +2841,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2851,7 +2851,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2861,7 +2861,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -3727,7 +3727,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__1</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3737,7 +3737,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3749,12 +3749,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__2</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__1</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3769,17 +3769,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__3</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__2</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3791,17 +3791,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__4</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__3</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3818,12 +3818,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__4</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -4375,7 +4375,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__1</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4385,7 +4385,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4397,12 +4397,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__2</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__1</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -4417,17 +4417,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__3</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__2</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -4439,17 +4439,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__4</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__3</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -4466,12 +4466,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__4</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -4807,7 +4807,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__1</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4829,12 +4829,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__2</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__1</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -4849,17 +4849,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__3</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__2</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4871,17 +4871,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__4</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__3</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4898,12 +4898,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__4</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">

</xml_diff>

<commit_message>
Fix IZZ/Refugee naming consistency and guard visualize edge cases (#171)
</commit_message>
<xml_diff>
--- a/src/vlinder/data/IZZ/xlsx/IZZ.xlsx
+++ b/src/vlinder/data/IZZ/xlsx/IZZ.xlsx
@@ -2431,7 +2431,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2441,7 +2441,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2451,7 +2451,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2461,7 +2461,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2631,7 +2631,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2641,7 +2641,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2651,7 +2651,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2661,7 +2661,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -2831,7 +2831,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2841,7 +2841,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2851,7 +2851,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2861,7 +2861,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -3727,7 +3727,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__1</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3737,7 +3737,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3749,12 +3749,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__2</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__1</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3769,17 +3769,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__3</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__2</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3791,17 +3791,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__4</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__3</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3818,12 +3818,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__4</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeDecreaseAbsenteeism_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -4375,7 +4375,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__1</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4385,7 +4385,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4397,12 +4397,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__2</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__1</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -4417,17 +4417,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__3</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__2</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -4439,17 +4439,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__4</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__3</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -4466,12 +4466,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__4</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeDecreaseStaffTurnover_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -4807,7 +4807,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__1</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__saturationpoint</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_saturationpoint</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4829,12 +4829,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__2</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__1</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_1</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -4849,17 +4849,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__3</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__2</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_2</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__accessiblepopulation</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_accessiblepopulation</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4871,17 +4871,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__4</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__3</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_3</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__probabilityofsuccess</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_probabilityofsuccess</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4898,12 +4898,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__4</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_4</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction__maximumeffect</t>
+          <t>RelativeIncreaseEmployeeSatisfaction_PhysicalStrainReduction_maximumeffect</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">

</xml_diff>